<commit_message>
Phase7-9: 平衡回归(bossMult r25 1.68→1.72回压0.3pp超沿; 终验N=300×3=56.3/63.7/60.7带内; streak4p 75-76%; 时长7.9s超时0.1%; 22哨兵N=100无>10pp真实漂移(四禧/咒术N=200复测落回噪声带)); 浏览器冒烟3局; export+xlsx重生成; 精修报告tools/idle_refine_report.md
</commit_message>
<xml_diff>
--- a/虚拟棋战_棋子与羁绊_20260914.xlsx
+++ b/虚拟棋战_棋子与羁绊_20260914.xlsx
@@ -1025,7 +1025,7 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>紫藤突刺：瞬步到最远的敌人身边，对其造成 214% 攻击伤害，突进至最远的敌人，并永久获得 15% 吸血</t>
+          <t>紫藤突刺：瞬步到最远的敌人身边，对其造成 214% 攻击伤害，突进至最远的敌人，并永久获得 15% 吸血（专属暴击 20%/2.2×）</t>
         </is>
       </c>
     </row>
@@ -1385,7 +1385,7 @@
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>熊猫跃袭：瞬步到最远的敌人身边，对其造成 246% 攻击伤害，突进至最远的敌人；目标生命低于 35% 时追加 60% 斩杀伤害</t>
+          <t>熊猫跃袭：瞬步到最远的敌人身边，对其造成 246% 攻击伤害，突进至最远的敌人；目标生命低于 35% 时追加 60% 斩杀伤害（专属暴击 20%/2.5×）</t>
         </is>
       </c>
     </row>
@@ -1475,7 +1475,7 @@
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>月影斩：瞬步到最远的敌人身边，对其造成 282% 攻击伤害，并附加每 3 秒 2% 最大生命的毒伤</t>
+          <t>月影斩：瞬步到最远的敌人身边，对其造成 282% 攻击伤害，并附加每 3 秒 2% 最大生命的毒伤（专属暴击 15%/2.2×）</t>
         </is>
       </c>
     </row>

</xml_diff>